<commit_message>
tweak damage ranges, adjust ptr and scar47
</commit_message>
<xml_diff>
--- a/changes/762x39-muzzles.xlsx
+++ b/changes/762x39-muzzles.xlsx
@@ -8,14 +8,27 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yifan\Documents\deadline-balancing\changes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6E2D15F2-0652-49E6-B0EE-DFFBE40E18C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2FD809E-A5FC-4CAC-9578-68C6E6546678}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{5142C438-6C5D-47F8-BFBE-C459086CFFFB}"/>
   </bookViews>
   <sheets>
     <sheet name="762x39-muzzles" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -1358,7 +1371,7 @@
         <v>-0.05</v>
       </c>
       <c r="I11">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="J11">
         <v>120</v>
@@ -1368,7 +1381,7 @@
       </c>
       <c r="N11">
         <f>C11-D11*20-E11*0.8-F11*0.6-H11*5+I11*15+J11/200</f>
-        <v>12.6</v>
+        <v>12.75</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
@@ -1430,7 +1443,7 @@
         <v>0.15</v>
       </c>
       <c r="I14">
-        <v>-0.01</v>
+        <v>0</v>
       </c>
       <c r="J14">
         <v>-30</v>
@@ -1440,7 +1453,7 @@
       </c>
       <c r="N14">
         <f>C14-D14*20-E14*0.8-F14*0.6-H14*5+I14*15+J14/200</f>
-        <v>-5.4500000000000011</v>
+        <v>-5.3000000000000007</v>
       </c>
     </row>
   </sheetData>

</xml_diff>